<commit_message>
Update attendees for quiz: flowable-enterprise — chinnadurai7608@gmail.com
</commit_message>
<xml_diff>
--- a/quizzes/flowable-enterprise/attendees.xlsx
+++ b/quizzes/flowable-enterprise/attendees.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M1"/>
+  <dimension ref="A1:M2"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -455,9 +455,50 @@
         <v>Grade</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>chinnadurai7608@gmail.com</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Chinnadurai P</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Flowable Enterprise</v>
+      </c>
+      <c r="D2" t="str">
+        <v>8/10/2026, 2:57:05 PM</v>
+      </c>
+      <c r="E2">
+        <v>25</v>
+      </c>
+      <c r="F2">
+        <v>25</v>
+      </c>
+      <c r="G2">
+        <v>25</v>
+      </c>
+      <c r="H2">
+        <v>0</v>
+      </c>
+      <c r="I2">
+        <v>0</v>
+      </c>
+      <c r="J2">
+        <v>25</v>
+      </c>
+      <c r="K2">
+        <v>25</v>
+      </c>
+      <c r="L2" t="str">
+        <v>100.00</v>
+      </c>
+      <c r="M2" t="str">
+        <v>A+</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M2"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update attendees for quiz: flowable-enterprise — vivekkumarsps@clarium.tech
</commit_message>
<xml_diff>
--- a/quizzes/flowable-enterprise/attendees.xlsx
+++ b/quizzes/flowable-enterprise/attendees.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M2"/>
+  <dimension ref="A1:M3"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -496,9 +496,50 @@
         <v>A+</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>vivekkumarsps@clarium.tech</v>
+      </c>
+      <c r="B3" t="str">
+        <v>vivek kumar</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Flowable Enterprise</v>
+      </c>
+      <c r="D3" t="str">
+        <v>8/12/2026, 3:14:12 PM</v>
+      </c>
+      <c r="E3">
+        <v>25</v>
+      </c>
+      <c r="F3">
+        <v>25</v>
+      </c>
+      <c r="G3">
+        <v>17</v>
+      </c>
+      <c r="H3">
+        <v>8</v>
+      </c>
+      <c r="I3">
+        <v>0</v>
+      </c>
+      <c r="J3">
+        <v>25</v>
+      </c>
+      <c r="K3">
+        <v>17</v>
+      </c>
+      <c r="L3" t="str">
+        <v>68.00</v>
+      </c>
+      <c r="M3" t="str">
+        <v>C</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update attendees for quiz: flowable-enterprise — bharathm@clarium.tech
</commit_message>
<xml_diff>
--- a/quizzes/flowable-enterprise/attendees.xlsx
+++ b/quizzes/flowable-enterprise/attendees.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M3"/>
+  <dimension ref="A1:M4"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -537,9 +537,50 @@
         <v>C</v>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>bharathm@clarium.tech</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Bharath</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Flowable Enterprise</v>
+      </c>
+      <c r="D4" t="str">
+        <v>8/12/2026, 3:16:20 PM</v>
+      </c>
+      <c r="E4">
+        <v>25</v>
+      </c>
+      <c r="F4">
+        <v>25</v>
+      </c>
+      <c r="G4">
+        <v>24</v>
+      </c>
+      <c r="H4">
+        <v>1</v>
+      </c>
+      <c r="I4">
+        <v>0</v>
+      </c>
+      <c r="J4">
+        <v>25</v>
+      </c>
+      <c r="K4">
+        <v>24</v>
+      </c>
+      <c r="L4" t="str">
+        <v>96.00</v>
+      </c>
+      <c r="M4" t="str">
+        <v>A+</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M4"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update attendees for quiz: flowable-enterprise — nirmalnarayanang@clarium.tech
</commit_message>
<xml_diff>
--- a/quizzes/flowable-enterprise/attendees.xlsx
+++ b/quizzes/flowable-enterprise/attendees.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M4"/>
+  <dimension ref="A1:M5"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -578,9 +578,50 @@
         <v>A+</v>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>nirmalnarayanang@clarium.tech</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Nirmal Narayanan</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Flowable Enterprise</v>
+      </c>
+      <c r="D5" t="str">
+        <v>8/12/2026, 3:16:55 PM</v>
+      </c>
+      <c r="E5">
+        <v>25</v>
+      </c>
+      <c r="F5">
+        <v>25</v>
+      </c>
+      <c r="G5">
+        <v>22</v>
+      </c>
+      <c r="H5">
+        <v>3</v>
+      </c>
+      <c r="I5">
+        <v>0</v>
+      </c>
+      <c r="J5">
+        <v>25</v>
+      </c>
+      <c r="K5">
+        <v>22</v>
+      </c>
+      <c r="L5" t="str">
+        <v>88.00</v>
+      </c>
+      <c r="M5" t="str">
+        <v>A</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M5"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update attendees for quiz: flowable-enterprise — asmithap@clarium.tech
</commit_message>
<xml_diff>
--- a/quizzes/flowable-enterprise/attendees.xlsx
+++ b/quizzes/flowable-enterprise/attendees.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M5"/>
+  <dimension ref="A1:M6"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -619,9 +619,50 @@
         <v>A</v>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>asmithap@clarium.tech</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Asmitha Singh</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Flowable Enterprise</v>
+      </c>
+      <c r="D6" t="str">
+        <v>8/12/2026, 3:17:18 PM</v>
+      </c>
+      <c r="E6">
+        <v>25</v>
+      </c>
+      <c r="F6">
+        <v>25</v>
+      </c>
+      <c r="G6">
+        <v>22</v>
+      </c>
+      <c r="H6">
+        <v>3</v>
+      </c>
+      <c r="I6">
+        <v>0</v>
+      </c>
+      <c r="J6">
+        <v>25</v>
+      </c>
+      <c r="K6">
+        <v>22</v>
+      </c>
+      <c r="L6" t="str">
+        <v>88.00</v>
+      </c>
+      <c r="M6" t="str">
+        <v>A</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M6"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update attendees for quiz: flowable-enterprise — nobelfranklinl@clarium.tech
</commit_message>
<xml_diff>
--- a/quizzes/flowable-enterprise/attendees.xlsx
+++ b/quizzes/flowable-enterprise/attendees.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M6"/>
+  <dimension ref="A1:M7"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -660,9 +660,50 @@
         <v>A</v>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>nobelfranklinl@clarium.tech</v>
+      </c>
+      <c r="B7" t="str">
+        <v>nobel franklin</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Flowable Enterprise</v>
+      </c>
+      <c r="D7" t="str">
+        <v>8/12/2026, 3:22:02 PM</v>
+      </c>
+      <c r="E7">
+        <v>25</v>
+      </c>
+      <c r="F7">
+        <v>25</v>
+      </c>
+      <c r="G7">
+        <v>22</v>
+      </c>
+      <c r="H7">
+        <v>3</v>
+      </c>
+      <c r="I7">
+        <v>0</v>
+      </c>
+      <c r="J7">
+        <v>25</v>
+      </c>
+      <c r="K7">
+        <v>22</v>
+      </c>
+      <c r="L7" t="str">
+        <v>88.00</v>
+      </c>
+      <c r="M7" t="str">
+        <v>A</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M7"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update attendees for quiz: flowable-enterprise — sanepayiabdullateefmp@clarium.tech
</commit_message>
<xml_diff>
--- a/quizzes/flowable-enterprise/attendees.xlsx
+++ b/quizzes/flowable-enterprise/attendees.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M7"/>
+  <dimension ref="A1:M8"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -466,7 +466,7 @@
         <v>Flowable Enterprise</v>
       </c>
       <c r="D2" t="str">
-        <v>8/10/2026, 2:57:05 PM</v>
+        <v>10/8/2026, 2:57:05 pm</v>
       </c>
       <c r="E2">
         <v>25</v>
@@ -507,7 +507,7 @@
         <v>Flowable Enterprise</v>
       </c>
       <c r="D3" t="str">
-        <v>8/12/2026, 3:14:12 PM</v>
+        <v>12/8/2026, 3:14:12 pm</v>
       </c>
       <c r="E3">
         <v>25</v>
@@ -548,7 +548,7 @@
         <v>Flowable Enterprise</v>
       </c>
       <c r="D4" t="str">
-        <v>8/12/2026, 3:16:20 PM</v>
+        <v>12/8/2026, 3:16:20 pm</v>
       </c>
       <c r="E4">
         <v>25</v>
@@ -589,7 +589,7 @@
         <v>Flowable Enterprise</v>
       </c>
       <c r="D5" t="str">
-        <v>8/12/2026, 3:16:55 PM</v>
+        <v>12/8/2026, 3:16:55 pm</v>
       </c>
       <c r="E5">
         <v>25</v>
@@ -630,7 +630,7 @@
         <v>Flowable Enterprise</v>
       </c>
       <c r="D6" t="str">
-        <v>8/12/2026, 3:17:18 PM</v>
+        <v>12/8/2026, 3:17:18 pm</v>
       </c>
       <c r="E6">
         <v>25</v>
@@ -671,7 +671,7 @@
         <v>Flowable Enterprise</v>
       </c>
       <c r="D7" t="str">
-        <v>8/12/2026, 3:22:02 PM</v>
+        <v>12/8/2026, 3:22:02 pm</v>
       </c>
       <c r="E7">
         <v>25</v>
@@ -698,12 +698,53 @@
         <v>88.00</v>
       </c>
       <c r="M7" t="str">
+        <v>A</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>sanepayiabdullateefmp@clarium.tech</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Abdul Lateef</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Flowable Enterprise</v>
+      </c>
+      <c r="D8" t="str">
+        <v>12/8/2026, 3:23:41 pm</v>
+      </c>
+      <c r="E8">
+        <v>25</v>
+      </c>
+      <c r="F8">
+        <v>25</v>
+      </c>
+      <c r="G8">
+        <v>21</v>
+      </c>
+      <c r="H8">
+        <v>4</v>
+      </c>
+      <c r="I8">
+        <v>0</v>
+      </c>
+      <c r="J8">
+        <v>25</v>
+      </c>
+      <c r="K8">
+        <v>21</v>
+      </c>
+      <c r="L8" t="str">
+        <v>84.00</v>
+      </c>
+      <c r="M8" t="str">
         <v>A</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M8"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update attendees for quiz: flowable-enterprise — kesavanm@clarium.tech
</commit_message>
<xml_diff>
--- a/quizzes/flowable-enterprise/attendees.xlsx
+++ b/quizzes/flowable-enterprise/attendees.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M8"/>
+  <dimension ref="A1:M9"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -466,7 +466,7 @@
         <v>Flowable Enterprise</v>
       </c>
       <c r="D2" t="str">
-        <v>10/8/2026, 2:57:05 pm</v>
+        <v>10/8/2026, 2:57:05 PM</v>
       </c>
       <c r="E2">
         <v>25</v>
@@ -507,7 +507,7 @@
         <v>Flowable Enterprise</v>
       </c>
       <c r="D3" t="str">
-        <v>12/8/2026, 3:14:12 pm</v>
+        <v>12/8/2026, 3:14:12 PM</v>
       </c>
       <c r="E3">
         <v>25</v>
@@ -548,7 +548,7 @@
         <v>Flowable Enterprise</v>
       </c>
       <c r="D4" t="str">
-        <v>12/8/2026, 3:16:20 pm</v>
+        <v>12/8/2026, 3:16:20 PM</v>
       </c>
       <c r="E4">
         <v>25</v>
@@ -589,7 +589,7 @@
         <v>Flowable Enterprise</v>
       </c>
       <c r="D5" t="str">
-        <v>12/8/2026, 3:16:55 pm</v>
+        <v>12/8/2026, 3:16:55 PM</v>
       </c>
       <c r="E5">
         <v>25</v>
@@ -630,7 +630,7 @@
         <v>Flowable Enterprise</v>
       </c>
       <c r="D6" t="str">
-        <v>12/8/2026, 3:17:18 pm</v>
+        <v>12/8/2026, 3:17:18 PM</v>
       </c>
       <c r="E6">
         <v>25</v>
@@ -671,7 +671,7 @@
         <v>Flowable Enterprise</v>
       </c>
       <c r="D7" t="str">
-        <v>12/8/2026, 3:22:02 pm</v>
+        <v>12/8/2026, 3:22:02 PM</v>
       </c>
       <c r="E7">
         <v>25</v>
@@ -712,7 +712,7 @@
         <v>Flowable Enterprise</v>
       </c>
       <c r="D8" t="str">
-        <v>12/8/2026, 3:23:41 pm</v>
+        <v>12/8/2026, 3:23:41 PM</v>
       </c>
       <c r="E8">
         <v>25</v>
@@ -742,9 +742,50 @@
         <v>A</v>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>kesavanm@clarium.tech</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Kesavan M</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Flowable Enterprise</v>
+      </c>
+      <c r="D9" t="str">
+        <v>8/12/2026, 3:24:54 PM</v>
+      </c>
+      <c r="E9">
+        <v>25</v>
+      </c>
+      <c r="F9">
+        <v>25</v>
+      </c>
+      <c r="G9">
+        <v>24</v>
+      </c>
+      <c r="H9">
+        <v>1</v>
+      </c>
+      <c r="I9">
+        <v>0</v>
+      </c>
+      <c r="J9">
+        <v>25</v>
+      </c>
+      <c r="K9">
+        <v>24</v>
+      </c>
+      <c r="L9" t="str">
+        <v>96.00</v>
+      </c>
+      <c r="M9" t="str">
+        <v>A+</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M9"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update attendees for quiz: flowable-enterprise — manirajav@clarium.tech
</commit_message>
<xml_diff>
--- a/quizzes/flowable-enterprise/attendees.xlsx
+++ b/quizzes/flowable-enterprise/attendees.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M9"/>
+  <dimension ref="A1:M10"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -783,9 +783,50 @@
         <v>A+</v>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>manirajav@clarium.tech</v>
+      </c>
+      <c r="B10" t="str">
+        <v>MANI RAJA V</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Flowable Enterprise</v>
+      </c>
+      <c r="D10" t="str">
+        <v>8/12/2026, 3:25:20 PM</v>
+      </c>
+      <c r="E10">
+        <v>25</v>
+      </c>
+      <c r="F10">
+        <v>25</v>
+      </c>
+      <c r="G10">
+        <v>23</v>
+      </c>
+      <c r="H10">
+        <v>2</v>
+      </c>
+      <c r="I10">
+        <v>0</v>
+      </c>
+      <c r="J10">
+        <v>25</v>
+      </c>
+      <c r="K10">
+        <v>23</v>
+      </c>
+      <c r="L10" t="str">
+        <v>92.00</v>
+      </c>
+      <c r="M10" t="str">
+        <v>A+</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M9"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M10"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update attendees for quiz: flowable-enterprise — fevinfm@clarium.tech
</commit_message>
<xml_diff>
--- a/quizzes/flowable-enterprise/attendees.xlsx
+++ b/quizzes/flowable-enterprise/attendees.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M10"/>
+  <dimension ref="A1:M11"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -824,9 +824,50 @@
         <v>A+</v>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>fevinfm@clarium.tech</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Fevin FM</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Flowable Enterprise</v>
+      </c>
+      <c r="D11" t="str">
+        <v>8/12/2026, 3:26:16 PM</v>
+      </c>
+      <c r="E11">
+        <v>25</v>
+      </c>
+      <c r="F11">
+        <v>25</v>
+      </c>
+      <c r="G11">
+        <v>23</v>
+      </c>
+      <c r="H11">
+        <v>2</v>
+      </c>
+      <c r="I11">
+        <v>0</v>
+      </c>
+      <c r="J11">
+        <v>25</v>
+      </c>
+      <c r="K11">
+        <v>23</v>
+      </c>
+      <c r="L11" t="str">
+        <v>92.00</v>
+      </c>
+      <c r="M11" t="str">
+        <v>A+</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M10"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M11"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update attendees for quiz: flowable-enterprise — krishnavenikb@clarium.tech
</commit_message>
<xml_diff>
--- a/quizzes/flowable-enterprise/attendees.xlsx
+++ b/quizzes/flowable-enterprise/attendees.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M11"/>
+  <dimension ref="A1:M12"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -865,9 +865,50 @@
         <v>A+</v>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>krishnavenikb@clarium.tech</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Krishanveni Katikala</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Flowable Enterprise</v>
+      </c>
+      <c r="D12" t="str">
+        <v>8/12/2026, 3:27:12 PM</v>
+      </c>
+      <c r="E12">
+        <v>25</v>
+      </c>
+      <c r="F12">
+        <v>25</v>
+      </c>
+      <c r="G12">
+        <v>24</v>
+      </c>
+      <c r="H12">
+        <v>1</v>
+      </c>
+      <c r="I12">
+        <v>0</v>
+      </c>
+      <c r="J12">
+        <v>25</v>
+      </c>
+      <c r="K12">
+        <v>24</v>
+      </c>
+      <c r="L12" t="str">
+        <v>96.00</v>
+      </c>
+      <c r="M12" t="str">
+        <v>A+</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M12"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update attendees for quiz: flowable-enterprise — gantasaisirriishaas@clarium.tech
</commit_message>
<xml_diff>
--- a/quizzes/flowable-enterprise/attendees.xlsx
+++ b/quizzes/flowable-enterprise/attendees.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M12"/>
+  <dimension ref="A1:M13"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -466,7 +466,7 @@
         <v>Flowable Enterprise</v>
       </c>
       <c r="D2" t="str">
-        <v>10/8/2026, 2:57:05 PM</v>
+        <v>8/10/2026, 2:57:05 pm</v>
       </c>
       <c r="E2">
         <v>25</v>
@@ -507,7 +507,7 @@
         <v>Flowable Enterprise</v>
       </c>
       <c r="D3" t="str">
-        <v>12/8/2026, 3:14:12 PM</v>
+        <v>8/12/2026, 3:14:12 pm</v>
       </c>
       <c r="E3">
         <v>25</v>
@@ -548,7 +548,7 @@
         <v>Flowable Enterprise</v>
       </c>
       <c r="D4" t="str">
-        <v>12/8/2026, 3:16:20 PM</v>
+        <v>8/12/2026, 3:16:20 pm</v>
       </c>
       <c r="E4">
         <v>25</v>
@@ -589,7 +589,7 @@
         <v>Flowable Enterprise</v>
       </c>
       <c r="D5" t="str">
-        <v>12/8/2026, 3:16:55 PM</v>
+        <v>8/12/2026, 3:16:55 pm</v>
       </c>
       <c r="E5">
         <v>25</v>
@@ -630,7 +630,7 @@
         <v>Flowable Enterprise</v>
       </c>
       <c r="D6" t="str">
-        <v>12/8/2026, 3:17:18 PM</v>
+        <v>8/12/2026, 3:17:18 pm</v>
       </c>
       <c r="E6">
         <v>25</v>
@@ -671,7 +671,7 @@
         <v>Flowable Enterprise</v>
       </c>
       <c r="D7" t="str">
-        <v>12/8/2026, 3:22:02 PM</v>
+        <v>8/12/2026, 3:22:02 pm</v>
       </c>
       <c r="E7">
         <v>25</v>
@@ -712,7 +712,7 @@
         <v>Flowable Enterprise</v>
       </c>
       <c r="D8" t="str">
-        <v>12/8/2026, 3:23:41 PM</v>
+        <v>8/12/2026, 3:23:41 pm</v>
       </c>
       <c r="E8">
         <v>25</v>
@@ -753,7 +753,7 @@
         <v>Flowable Enterprise</v>
       </c>
       <c r="D9" t="str">
-        <v>8/12/2026, 3:24:54 PM</v>
+        <v>12/8/2026, 3:24:54 pm</v>
       </c>
       <c r="E9">
         <v>25</v>
@@ -794,7 +794,7 @@
         <v>Flowable Enterprise</v>
       </c>
       <c r="D10" t="str">
-        <v>8/12/2026, 3:25:20 PM</v>
+        <v>12/8/2026, 3:25:20 pm</v>
       </c>
       <c r="E10">
         <v>25</v>
@@ -835,7 +835,7 @@
         <v>Flowable Enterprise</v>
       </c>
       <c r="D11" t="str">
-        <v>8/12/2026, 3:26:16 PM</v>
+        <v>12/8/2026, 3:26:16 pm</v>
       </c>
       <c r="E11">
         <v>25</v>
@@ -876,7 +876,7 @@
         <v>Flowable Enterprise</v>
       </c>
       <c r="D12" t="str">
-        <v>8/12/2026, 3:27:12 PM</v>
+        <v>12/8/2026, 3:27:12 pm</v>
       </c>
       <c r="E12">
         <v>25</v>
@@ -906,9 +906,50 @@
         <v>A+</v>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>gantasaisirriishaas@clarium.tech</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Ganta Sai Sirriisha</v>
+      </c>
+      <c r="C13" t="str">
+        <v>Flowable Enterprise</v>
+      </c>
+      <c r="D13" t="str">
+        <v>12/8/2026, 3:28:24 pm</v>
+      </c>
+      <c r="E13">
+        <v>25</v>
+      </c>
+      <c r="F13">
+        <v>25</v>
+      </c>
+      <c r="G13">
+        <v>23</v>
+      </c>
+      <c r="H13">
+        <v>2</v>
+      </c>
+      <c r="I13">
+        <v>0</v>
+      </c>
+      <c r="J13">
+        <v>25</v>
+      </c>
+      <c r="K13">
+        <v>23</v>
+      </c>
+      <c r="L13" t="str">
+        <v>92.00</v>
+      </c>
+      <c r="M13" t="str">
+        <v>A+</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M12"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M13"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>